<commit_message>
Updated power sector files for RPS date + utility and distributed solar additions based on data files from NEXT Group.
</commit_message>
<xml_diff>
--- a/InputData/elec/BRPSDbS/BAU RPS Data by Subregion.xlsx
+++ b/InputData/elec/BRPSDbS/BAU RPS Data by Subregion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\South Korea\Models\eps-southkorea\InputData\elec\BRPSDbS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1EB2F35-95E1-433C-8DAA-59C590888467}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26881B1B-E315-45FF-84CB-456DA879815C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="465" yWindow="795" windowWidth="25770" windowHeight="20955" tabRatio="787" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1520" yWindow="1520" windowWidth="28800" windowHeight="15450" tabRatio="787" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -1466,13 +1466,13 @@
     <t>BAU CES switch (1 = CES in BAU, 0 = removed). 2026-09-14: set to 0 - partner round 2 decision: the 11th Plan buildout is already in BPMCCS, so a BAU CES double counts; CES becomes a policy lever. Rows 3-8 kept for reference.</t>
   </si>
   <si>
-    <t>RPS abolition year (partner round 2, 2026-09-11: requirement set to 0 from the year the RPS is abolished and replaced by government-set auction volumes; later renewables enter via the RPS/auction policy levers). YEAR IS AN ASSUMPTION pending partner confirmation - change B19 only.</t>
-  </si>
-  <si>
     <t>RPS REQUIREMENT USED IN THE OUTPUT FILE (= row 15, 0 from the abolition year)</t>
   </si>
   <si>
-    <t>2026-09-14 partner round 2: (1) CES removed from the BAU - CES_kor!B10 switch = 0 multiplies the CES output row, so BRPSDbS-CES-percentages is all zeros (partner confirmed a zero-CES run converges to the mandated capacity; the 11th Plan buildout in BPMCCS would otherwise be double counted). (2) RPS requirement set to 0 from the RPS abolition year (RPS_basis!B19, ASSUMED 2027 pending partner confirmation) via RPS_basis row 20; 2021-2026 keep the rebased legal ratio. Neither change moves BAU results: the RPS credit price was already 0 in every year, and the CES only bound at the cap in 2021-25 and mildly in 2030-35 (~3 GW solar).</t>
+    <t>RPS abolition year (partner round 2/3, confirmed 2026-09-15: REC issuance for new facilities ends in 2027 under the legislative reform, new projects move to long-term fixed-price contracts; the existing-facility REC market runs to end-2029 under transitional rules, but zeroing the requirement from 2027 is most consistent with the reform). Requirement = 0 from this year; later renewables enter via the RPS/auction policy levers. Change B19 only.</t>
+  </si>
+  <si>
+    <t>2026-09-14 partner round 2: (1) CES removed from the BAU - CES_kor!B10 switch = 0 multiplies the CES output row, so BRPSDbS-CES-percentages is all zeros (partner confirmed a zero-CES run converges to the mandated capacity; the 11th Plan buildout in BPMCCS would otherwise be double counted). (2) RPS requirement set to 0 from the RPS abolition year (RPS_basis!B19, 2027, confirmed by the partner 2026-09-15: new-facility REC issuance ends 2027) via RPS_basis row 20; 2021-2026 keep the rebased legal ratio. Neither change moves BAU results: the RPS credit price was already 0 in every year, and the CES only bound at the cap in 2021-25 and mildly in 2030-35 (~3 GW solar).</t>
   </si>
 </sst>
 </file>
@@ -2799,58 +2799,22 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="51"/>
-    <xf numFmtId="0" fontId="27" fillId="43" borderId="36" xfId="54" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="36" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="34" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="36" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="34" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="36" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="36" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="36" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="36" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="36" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="36" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="36" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="36" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="36" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="19" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="36" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2880,22 +2844,58 @@
     <xf numFmtId="0" fontId="32" fillId="36" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="34" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="19" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="34" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="43" borderId="36" xfId="54" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="36" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="36" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="36" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="36" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="36" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="36" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="36" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="36" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="36" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="36" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="36" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="35" borderId="1" xfId="54" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3379,10 +3379,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B60"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="122.7109375" customWidth="1"/>
+    <col min="2" max="2" width="122.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -3395,7 +3395,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="17.100000000000001" customHeight="1">
+    <row r="3" spans="1:2" ht="17.149999999999999" customHeight="1">
       <c r="A3" s="1" t="s">
         <v>317</v>
       </c>
@@ -3629,16 +3629,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58D2CBCD-AD0F-4CC9-AC7B-9D4067D1C400}">
   <dimension ref="A1:I82"/>
-  <sheetFormatPr defaultColWidth="20.5703125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="20.54296875" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="33.7109375" style="13" customWidth="1"/>
-    <col min="2" max="2" width="13.140625" style="13" customWidth="1"/>
-    <col min="3" max="3" width="8.7109375" style="13" customWidth="1"/>
+    <col min="1" max="1" width="33.7265625" style="13" customWidth="1"/>
+    <col min="2" max="2" width="13.1796875" style="13" customWidth="1"/>
+    <col min="3" max="3" width="8.7265625" style="13" customWidth="1"/>
     <col min="4" max="4" width="8" style="13" customWidth="1"/>
-    <col min="5" max="16384" width="20.5703125" style="13"/>
+    <col min="5" max="16384" width="20.54296875" style="13"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="1" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A1" s="26" t="s">
         <v>321</v>
       </c>
@@ -3667,7 +3667,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="2" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A2" s="28" t="s">
         <v>325</v>
       </c>
@@ -3696,7 +3696,7 @@
         <v>637103809</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="3" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A3" s="30" t="s">
         <v>170</v>
       </c>
@@ -3725,7 +3725,7 @@
         <v>4677237</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="4" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A4" s="28" t="s">
         <v>328</v>
       </c>
@@ -3754,7 +3754,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="5" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A5" s="30" t="s">
         <v>170</v>
       </c>
@@ -3783,7 +3783,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="6" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A6" s="30" t="s">
         <v>170</v>
       </c>
@@ -3812,7 +3812,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="7" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A7" s="28" t="s">
         <v>330</v>
       </c>
@@ -3841,7 +3841,7 @@
         <v>68115782</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="8" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A8" s="30" t="s">
         <v>170</v>
       </c>
@@ -3870,7 +3870,7 @@
         <v>62487770</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="9" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A9" s="30" t="s">
         <v>170</v>
       </c>
@@ -3899,7 +3899,7 @@
         <v>5628012</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="10" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A10" s="30" t="s">
         <v>170</v>
       </c>
@@ -3928,7 +3928,7 @@
         <v>58460649</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="11" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A11" s="30" t="s">
         <v>170</v>
       </c>
@@ -3957,7 +3957,7 @@
         <v>52953466</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="12" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A12" s="30" t="s">
         <v>170</v>
       </c>
@@ -3986,7 +3986,7 @@
         <v>5507183</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="13" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A13" s="30" t="s">
         <v>170</v>
       </c>
@@ -4015,7 +4015,7 @@
         <v>9655133</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="14" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A14" s="30" t="s">
         <v>170</v>
       </c>
@@ -4044,7 +4044,7 @@
         <v>9534304</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="15" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A15" s="30" t="s">
         <v>170</v>
       </c>
@@ -4073,7 +4073,7 @@
         <v>120828</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="16" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A16" s="28" t="s">
         <v>335</v>
       </c>
@@ -4102,7 +4102,7 @@
         <v>37449731</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="17" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A17" s="30" t="s">
         <v>170</v>
       </c>
@@ -4131,7 +4131,7 @@
         <v>32334925</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="18" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A18" s="30" t="s">
         <v>170</v>
       </c>
@@ -4160,7 +4160,7 @@
         <v>5114806</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="19" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A19" s="30" t="s">
         <v>170</v>
       </c>
@@ -4189,7 +4189,7 @@
         <v>3736569</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="20" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A20" s="30" t="s">
         <v>170</v>
       </c>
@@ -4218,7 +4218,7 @@
         <v>3723163</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="21" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A21" s="30" t="s">
         <v>170</v>
       </c>
@@ -4247,7 +4247,7 @@
         <v>13406</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="22" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A22" s="30" t="s">
         <v>170</v>
       </c>
@@ -4276,7 +4276,7 @@
         <v>4313488</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="23" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A23" s="30" t="s">
         <v>170</v>
       </c>
@@ -4305,7 +4305,7 @@
         <v>4311955</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="24" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A24" s="30" t="s">
         <v>170</v>
       </c>
@@ -4334,7 +4334,7 @@
         <v>1532</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="25" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A25" s="30" t="s">
         <v>170</v>
       </c>
@@ -4363,7 +4363,7 @@
         <v>418483</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="26" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A26" s="30" t="s">
         <v>170</v>
       </c>
@@ -4392,7 +4392,7 @@
         <v>418483</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="27" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A27" s="30" t="s">
         <v>170</v>
       </c>
@@ -4421,7 +4421,7 @@
         <v>12117654</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="28" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A28" s="30" t="s">
         <v>170</v>
       </c>
@@ -4450,7 +4450,7 @@
         <v>11823889</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="29" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A29" s="30" t="s">
         <v>170</v>
       </c>
@@ -4479,7 +4479,7 @@
         <v>293765</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="30" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A30" s="30" t="s">
         <v>170</v>
       </c>
@@ -4508,7 +4508,7 @@
         <v>194068</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="31" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A31" s="30" t="s">
         <v>170</v>
       </c>
@@ -4537,7 +4537,7 @@
         <v>152244</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="32" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A32" s="30" t="s">
         <v>170</v>
       </c>
@@ -4566,7 +4566,7 @@
         <v>41823</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="33" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A33" s="30" t="s">
         <v>170</v>
       </c>
@@ -4595,7 +4595,7 @@
         <v>179394</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="34" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A34" s="30" t="s">
         <v>170</v>
       </c>
@@ -4624,7 +4624,7 @@
         <v>179394</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="35" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A35" s="30" t="s">
         <v>170</v>
       </c>
@@ -4653,7 +4653,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="36" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A36" s="30" t="s">
         <v>170</v>
       </c>
@@ -4682,7 +4682,7 @@
         <v>559688</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="37" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A37" s="30" t="s">
         <v>170</v>
       </c>
@@ -4711,7 +4711,7 @@
         <v>559688</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="38" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A38" s="30" t="s">
         <v>170</v>
       </c>
@@ -4740,7 +4740,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="39" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A39" s="30" t="s">
         <v>170</v>
       </c>
@@ -4769,7 +4769,7 @@
         <v>7245849</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="40" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A40" s="30" t="s">
         <v>170</v>
       </c>
@@ -4798,7 +4798,7 @@
         <v>7245849</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="41" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A41" s="30" t="s">
         <v>170</v>
       </c>
@@ -4827,7 +4827,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="42" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A42" s="30" t="s">
         <v>170</v>
       </c>
@@ -4856,7 +4856,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="43" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A43" s="30" t="s">
         <v>170</v>
       </c>
@@ -4885,7 +4885,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="44" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A44" s="30" t="s">
         <v>170</v>
       </c>
@@ -4914,7 +4914,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="45" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A45" s="30" t="s">
         <v>170</v>
       </c>
@@ -4943,7 +4943,7 @@
         <v>251942</v>
       </c>
     </row>
-    <row r="46" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="46" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A46" s="30" t="s">
         <v>170</v>
       </c>
@@ -4972,7 +4972,7 @@
         <v>251942</v>
       </c>
     </row>
-    <row r="47" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="47" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A47" s="30" t="s">
         <v>170</v>
       </c>
@@ -5001,7 +5001,7 @@
         <v>159149</v>
       </c>
     </row>
-    <row r="48" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="48" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A48" s="30" t="s">
         <v>170</v>
       </c>
@@ -5030,7 +5030,7 @@
         <v>159149</v>
       </c>
     </row>
-    <row r="49" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="49" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A49" s="30" t="s">
         <v>170</v>
       </c>
@@ -5059,7 +5059,7 @@
         <v>2159997</v>
       </c>
     </row>
-    <row r="50" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="50" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A50" s="30" t="s">
         <v>170</v>
       </c>
@@ -5088,7 +5088,7 @@
         <v>2159997</v>
       </c>
     </row>
-    <row r="51" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="51" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A51" s="30" t="s">
         <v>170</v>
       </c>
@@ -5117,7 +5117,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="52" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A52" s="30" t="s">
         <v>170</v>
       </c>
@@ -5146,7 +5146,7 @@
         <v>1367568</v>
       </c>
     </row>
-    <row r="53" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="53" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A53" s="30" t="s">
         <v>170</v>
       </c>
@@ -5175,7 +5175,7 @@
         <v>1367568</v>
       </c>
     </row>
-    <row r="54" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="54" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A54" s="30" t="s">
         <v>170</v>
       </c>
@@ -5204,7 +5204,7 @@
         <v>424724</v>
       </c>
     </row>
-    <row r="55" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="55" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A55" s="30" t="s">
         <v>170</v>
       </c>
@@ -5233,7 +5233,7 @@
         <v>341051</v>
       </c>
     </row>
-    <row r="56" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="56" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A56" s="30" t="s">
         <v>170</v>
       </c>
@@ -5262,7 +5262,7 @@
         <v>83673</v>
       </c>
     </row>
-    <row r="57" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="57" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A57" s="30" t="s">
         <v>170</v>
       </c>
@@ -5291,7 +5291,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="58" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="58" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A58" s="30" t="s">
         <v>170</v>
       </c>
@@ -5320,7 +5320,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="59" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="59" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A59" s="30" t="s">
         <v>170</v>
       </c>
@@ -5349,7 +5349,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="60" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="60" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A60" s="30" t="s">
         <v>170</v>
       </c>
@@ -5378,7 +5378,7 @@
         <v>91722</v>
       </c>
     </row>
-    <row r="61" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="61" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A61" s="30" t="s">
         <v>170</v>
       </c>
@@ -5407,7 +5407,7 @@
         <v>87605</v>
       </c>
     </row>
-    <row r="62" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="62" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A62" s="30" t="s">
         <v>170</v>
       </c>
@@ -5436,7 +5436,7 @@
         <v>4117</v>
       </c>
     </row>
-    <row r="63" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="63" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A63" s="30" t="s">
         <v>170</v>
       </c>
@@ -5465,7 +5465,7 @@
         <v>212389</v>
       </c>
     </row>
-    <row r="64" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="64" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A64" s="30" t="s">
         <v>170</v>
       </c>
@@ -5494,7 +5494,7 @@
         <v>132833</v>
       </c>
     </row>
-    <row r="65" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="65" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A65" s="30" t="s">
         <v>170</v>
       </c>
@@ -5523,7 +5523,7 @@
         <v>79556</v>
       </c>
     </row>
-    <row r="66" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="66" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A66" s="30" t="s">
         <v>170</v>
       </c>
@@ -5552,7 +5552,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="67" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="67" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A67" s="30" t="s">
         <v>170</v>
       </c>
@@ -5581,7 +5581,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="68" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="68" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A68" s="30" t="s">
         <v>170</v>
       </c>
@@ -5610,7 +5610,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="69" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="69" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A69" s="30" t="s">
         <v>170</v>
       </c>
@@ -5639,7 +5639,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="70" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="70" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A70" s="30" t="s">
         <v>170</v>
       </c>
@@ -5668,7 +5668,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="71" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="71" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A71" s="30" t="s">
         <v>170</v>
       </c>
@@ -5697,7 +5697,7 @@
         <v>120613</v>
       </c>
     </row>
-    <row r="72" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="72" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A72" s="30" t="s">
         <v>170</v>
       </c>
@@ -5726,7 +5726,7 @@
         <v>120613</v>
       </c>
     </row>
-    <row r="73" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="73" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A73" s="30" t="s">
         <v>170</v>
       </c>
@@ -5755,7 +5755,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="74" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A74" s="30" t="s">
         <v>170</v>
       </c>
@@ -5784,7 +5784,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="75" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A75" s="30" t="s">
         <v>170</v>
       </c>
@@ -5813,7 +5813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="76" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A76" s="30" t="s">
         <v>170</v>
       </c>
@@ -5842,7 +5842,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="77" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="77" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A77" s="30" t="s">
         <v>170</v>
       </c>
@@ -5871,7 +5871,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="78" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="78" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A78" s="28" t="s">
         <v>359</v>
       </c>
@@ -5900,7 +5900,7 @@
         <v>7583357</v>
       </c>
     </row>
-    <row r="79" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="79" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A79" s="30" t="s">
         <v>170</v>
       </c>
@@ -5929,7 +5929,7 @@
         <v>7462529</v>
       </c>
     </row>
-    <row r="80" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="80" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A80" s="30" t="s">
         <v>170</v>
       </c>
@@ -5958,7 +5958,7 @@
         <v>120828</v>
       </c>
     </row>
-    <row r="81" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="81" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A81" s="30" t="s">
         <v>170</v>
       </c>
@@ -5987,7 +5987,7 @@
         <v>2071775</v>
       </c>
     </row>
-    <row r="82" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="82" spans="1:9" ht="20.149999999999999" customHeight="1">
       <c r="A82" s="32" t="s">
         <v>170</v>
       </c>
@@ -6025,12 +6025,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7351AFFB-16B7-4DBB-8DC6-20B8594B3331}">
   <dimension ref="A3:H27"/>
-  <sheetFormatPr defaultColWidth="21" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="21" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="16384" width="21" style="13"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:8" ht="20.100000000000001" customHeight="1">
+    <row r="3" spans="1:8" ht="20.149999999999999" customHeight="1">
       <c r="A3" s="26" t="s">
         <v>321</v>
       </c>
@@ -6056,7 +6056,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="20.100000000000001" customHeight="1">
+    <row r="4" spans="1:8" ht="20.149999999999999" customHeight="1">
       <c r="A4" s="28" t="s">
         <v>316</v>
       </c>
@@ -6082,7 +6082,7 @@
         <v>595601</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="20.100000000000001" customHeight="1">
+    <row r="5" spans="1:8" ht="20.149999999999999" customHeight="1">
       <c r="A5" s="28" t="s">
         <v>171</v>
       </c>
@@ -6108,7 +6108,7 @@
         <v>188754</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="20.100000000000001" customHeight="1">
+    <row r="6" spans="1:8" ht="20.149999999999999" customHeight="1">
       <c r="A6" s="28" t="s">
         <v>364</v>
       </c>
@@ -6134,7 +6134,7 @@
         <v>335561</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="20.100000000000001" customHeight="1">
+    <row r="7" spans="1:8" ht="20.149999999999999" customHeight="1">
       <c r="A7" s="30" t="s">
         <v>170</v>
       </c>
@@ -6160,7 +6160,7 @@
         <v>167152</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="20.100000000000001" customHeight="1">
+    <row r="8" spans="1:8" ht="20.149999999999999" customHeight="1">
       <c r="A8" s="30" t="s">
         <v>170</v>
       </c>
@@ -6186,7 +6186,7 @@
         <v>165241</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="20.100000000000001" customHeight="1">
+    <row r="9" spans="1:8" ht="20.149999999999999" customHeight="1">
       <c r="A9" s="30" t="s">
         <v>170</v>
       </c>
@@ -6212,7 +6212,7 @@
         <v>1911</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="20.100000000000001" customHeight="1">
+    <row r="10" spans="1:8" ht="20.149999999999999" customHeight="1">
       <c r="A10" s="30" t="s">
         <v>170</v>
       </c>
@@ -6238,7 +6238,7 @@
         <v>1204</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="20.100000000000001" customHeight="1">
+    <row r="11" spans="1:8" ht="20.149999999999999" customHeight="1">
       <c r="A11" s="30" t="s">
         <v>170</v>
       </c>
@@ -6264,7 +6264,7 @@
         <v>167205</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="20.100000000000001" customHeight="1">
+    <row r="12" spans="1:8" ht="20.149999999999999" customHeight="1">
       <c r="A12" s="28" t="s">
         <v>175</v>
       </c>
@@ -6290,7 +6290,7 @@
         <v>4677</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="20.100000000000001" customHeight="1">
+    <row r="13" spans="1:8" ht="20.149999999999999" customHeight="1">
       <c r="A13" s="33" t="s">
         <v>367</v>
       </c>
@@ -6661,30 +6661,30 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6393E301-1DF3-46BD-A777-073878B6935A}">
   <dimension ref="A1:T81"/>
-  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="15.28515625" style="13" customWidth="1"/>
-    <col min="2" max="2" width="11.140625" style="13" customWidth="1"/>
-    <col min="3" max="3" width="16.42578125" style="13" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.28515625" style="13" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.42578125" style="13" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.28515625" style="13" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="15.28515625" style="13" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.140625" style="13" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.28515625" style="13" bestFit="1" customWidth="1"/>
-    <col min="11" max="17" width="8.5703125" style="13"/>
-    <col min="18" max="18" width="12.7109375" style="13" bestFit="1" customWidth="1"/>
-    <col min="19" max="16384" width="8.5703125" style="13"/>
+    <col min="1" max="1" width="15.26953125" style="13" customWidth="1"/>
+    <col min="2" max="2" width="11.1796875" style="13" customWidth="1"/>
+    <col min="3" max="3" width="16.453125" style="13" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.26953125" style="13" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.453125" style="13" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.26953125" style="13" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="15.26953125" style="13" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.1796875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.26953125" style="13" bestFit="1" customWidth="1"/>
+    <col min="11" max="17" width="8.54296875" style="13"/>
+    <col min="18" max="18" width="12.7265625" style="13" bestFit="1" customWidth="1"/>
+    <col min="19" max="16384" width="8.54296875" style="13"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20">
-      <c r="B1" s="96" t="s">
+      <c r="B1" s="117" t="s">
         <v>421</v>
       </c>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
       <c r="G1" s="66" t="s">
         <v>422</v>
       </c>
@@ -7422,56 +7422,56 @@
       <c r="E20" s="34"/>
       <c r="F20" s="34"/>
     </row>
-    <row r="21" spans="1:13" ht="17.100000000000001" customHeight="1">
-      <c r="A21" s="97" t="s">
+    <row r="21" spans="1:13" ht="17.149999999999999" customHeight="1">
+      <c r="A21" s="118" t="s">
         <v>379</v>
       </c>
-      <c r="B21" s="101" t="s">
+      <c r="B21" s="120" t="s">
         <v>380</v>
       </c>
-      <c r="C21" s="101" t="s">
+      <c r="C21" s="120" t="s">
         <v>371</v>
       </c>
-      <c r="D21" s="101" t="s">
+      <c r="D21" s="120" t="s">
         <v>372</v>
       </c>
-      <c r="E21" s="101" t="s">
+      <c r="E21" s="120" t="s">
         <v>173</v>
       </c>
-      <c r="F21" s="103" t="s">
+      <c r="F21" s="122" t="s">
         <v>373</v>
       </c>
-      <c r="G21" s="103" t="s">
+      <c r="G21" s="122" t="s">
         <v>381</v>
       </c>
-      <c r="H21" s="101" t="s">
+      <c r="H21" s="120" t="s">
         <v>382</v>
       </c>
-      <c r="I21" s="101" t="s">
+      <c r="I21" s="120" t="s">
         <v>376</v>
       </c>
-      <c r="J21" s="105" t="s">
+      <c r="J21" s="124" t="s">
         <v>370</v>
       </c>
       <c r="K21" s="17"/>
-      <c r="L21" s="107"/>
-      <c r="M21" s="107"/>
-    </row>
-    <row r="22" spans="1:13" ht="36">
-      <c r="A22" s="98"/>
-      <c r="B22" s="102"/>
-      <c r="C22" s="102"/>
-      <c r="D22" s="102"/>
-      <c r="E22" s="102"/>
-      <c r="F22" s="104"/>
-      <c r="G22" s="104"/>
-      <c r="H22" s="102"/>
-      <c r="I22" s="102"/>
-      <c r="J22" s="106"/>
-      <c r="K22" s="108" t="s">
+      <c r="L21" s="126"/>
+      <c r="M21" s="126"/>
+    </row>
+    <row r="22" spans="1:13" ht="35">
+      <c r="A22" s="119"/>
+      <c r="B22" s="121"/>
+      <c r="C22" s="121"/>
+      <c r="D22" s="121"/>
+      <c r="E22" s="121"/>
+      <c r="F22" s="123"/>
+      <c r="G22" s="123"/>
+      <c r="H22" s="121"/>
+      <c r="I22" s="121"/>
+      <c r="J22" s="125"/>
+      <c r="K22" s="127" t="s">
         <v>383</v>
       </c>
-      <c r="L22" s="109"/>
+      <c r="L22" s="128"/>
       <c r="M22" s="18" t="s">
         <v>384</v>
       </c>
@@ -7507,10 +7507,10 @@
       <c r="J23" s="21">
         <v>588</v>
       </c>
-      <c r="K23" s="99">
+      <c r="K23" s="113">
         <v>358.2</v>
       </c>
-      <c r="L23" s="100"/>
+      <c r="L23" s="114"/>
       <c r="M23" s="22">
         <v>229.9</v>
       </c>
@@ -7546,16 +7546,16 @@
       <c r="J24" s="24">
         <v>100</v>
       </c>
-      <c r="K24" s="112">
+      <c r="K24" s="115">
         <v>60.9</v>
       </c>
-      <c r="L24" s="113"/>
+      <c r="L24" s="116"/>
       <c r="M24" s="25">
         <v>39.1</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="17.649999999999999" customHeight="1">
-      <c r="A25" s="110" t="s">
+      <c r="A25" s="111" t="s">
         <v>410</v>
       </c>
       <c r="B25" s="20" t="s">
@@ -7585,16 +7585,16 @@
       <c r="J25" s="21">
         <v>642.6</v>
       </c>
-      <c r="K25" s="99">
+      <c r="K25" s="113">
         <v>302</v>
       </c>
-      <c r="L25" s="100"/>
+      <c r="L25" s="114"/>
       <c r="M25" s="22">
         <v>340.6</v>
       </c>
     </row>
     <row r="26" spans="1:13" ht="17.649999999999999" customHeight="1">
-      <c r="A26" s="111"/>
+      <c r="A26" s="112"/>
       <c r="B26" s="23" t="s">
         <v>378</v>
       </c>
@@ -7622,16 +7622,16 @@
       <c r="J26" s="24">
         <v>100</v>
       </c>
-      <c r="K26" s="112">
+      <c r="K26" s="115">
         <v>47</v>
       </c>
-      <c r="L26" s="113"/>
+      <c r="L26" s="116"/>
       <c r="M26" s="25">
         <v>53</v>
       </c>
     </row>
     <row r="27" spans="1:13" ht="17.649999999999999" customHeight="1">
-      <c r="A27" s="110" t="s">
+      <c r="A27" s="111" t="s">
         <v>411</v>
       </c>
       <c r="B27" s="20" t="s">
@@ -7661,16 +7661,16 @@
       <c r="J27" s="21">
         <v>691.5</v>
       </c>
-      <c r="K27" s="99">
+      <c r="K27" s="113">
         <v>242.8</v>
       </c>
-      <c r="L27" s="100"/>
+      <c r="L27" s="114"/>
       <c r="M27" s="22">
         <v>448.7</v>
       </c>
     </row>
     <row r="28" spans="1:13" ht="17.649999999999999" customHeight="1">
-      <c r="A28" s="111"/>
+      <c r="A28" s="112"/>
       <c r="B28" s="23" t="s">
         <v>378</v>
       </c>
@@ -7698,16 +7698,16 @@
       <c r="J28" s="24">
         <v>100</v>
       </c>
-      <c r="K28" s="112">
+      <c r="K28" s="115">
         <v>35.1</v>
       </c>
-      <c r="L28" s="113"/>
+      <c r="L28" s="116"/>
       <c r="M28" s="25">
         <v>64.900000000000006</v>
       </c>
     </row>
     <row r="29" spans="1:13" ht="17.649999999999999" customHeight="1">
-      <c r="A29" s="110" t="s">
+      <c r="A29" s="111" t="s">
         <v>412</v>
       </c>
       <c r="B29" s="20" t="s">
@@ -7737,16 +7737,16 @@
       <c r="J29" s="21">
         <v>704.5</v>
       </c>
-      <c r="K29" s="99">
+      <c r="K29" s="113">
         <v>206.7</v>
       </c>
-      <c r="L29" s="100"/>
+      <c r="L29" s="114"/>
       <c r="M29" s="22">
         <v>497.8</v>
       </c>
     </row>
     <row r="30" spans="1:13" ht="17.649999999999999" customHeight="1">
-      <c r="A30" s="111"/>
+      <c r="A30" s="112"/>
       <c r="B30" s="23" t="s">
         <v>378</v>
       </c>
@@ -7774,10 +7774,10 @@
       <c r="J30" s="24">
         <v>100</v>
       </c>
-      <c r="K30" s="112">
+      <c r="K30" s="115">
         <v>29.3</v>
       </c>
-      <c r="L30" s="113"/>
+      <c r="L30" s="116"/>
       <c r="M30" s="25">
         <v>70.7</v>
       </c>
@@ -7793,66 +7793,66 @@
       </c>
     </row>
     <row r="34" spans="1:20">
-      <c r="A34" s="114" t="s">
+      <c r="A34" s="102" t="s">
         <v>379</v>
       </c>
-      <c r="B34" s="117" t="s">
+      <c r="B34" s="105" t="s">
         <v>389</v>
       </c>
-      <c r="C34" s="118"/>
-      <c r="D34" s="118"/>
-      <c r="E34" s="118"/>
-      <c r="F34" s="118"/>
-      <c r="G34" s="118"/>
-      <c r="H34" s="118"/>
-      <c r="I34" s="118"/>
-      <c r="J34" s="118"/>
-      <c r="K34" s="119"/>
-      <c r="L34" s="120" t="s">
+      <c r="C34" s="106"/>
+      <c r="D34" s="106"/>
+      <c r="E34" s="106"/>
+      <c r="F34" s="106"/>
+      <c r="G34" s="106"/>
+      <c r="H34" s="106"/>
+      <c r="I34" s="106"/>
+      <c r="J34" s="106"/>
+      <c r="K34" s="107"/>
+      <c r="L34" s="108" t="s">
         <v>390</v>
       </c>
       <c r="M34" s="36" t="s">
         <v>370</v>
       </c>
     </row>
-    <row r="35" spans="1:20" ht="25.5">
-      <c r="A35" s="115"/>
-      <c r="B35" s="117" t="s">
+    <row r="35" spans="1:20">
+      <c r="A35" s="103"/>
+      <c r="B35" s="105" t="s">
         <v>391</v>
       </c>
-      <c r="C35" s="118"/>
-      <c r="D35" s="118"/>
-      <c r="E35" s="118"/>
-      <c r="F35" s="118"/>
-      <c r="G35" s="119"/>
-      <c r="H35" s="117" t="s">
+      <c r="C35" s="106"/>
+      <c r="D35" s="106"/>
+      <c r="E35" s="106"/>
+      <c r="F35" s="106"/>
+      <c r="G35" s="107"/>
+      <c r="H35" s="105" t="s">
         <v>381</v>
       </c>
-      <c r="I35" s="118"/>
-      <c r="J35" s="119"/>
+      <c r="I35" s="106"/>
+      <c r="J35" s="107"/>
       <c r="K35" s="35" t="s">
         <v>370</v>
       </c>
-      <c r="L35" s="121"/>
+      <c r="L35" s="109"/>
       <c r="M35" s="37" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="36" spans="1:20" ht="25.5">
-      <c r="A36" s="115"/>
-      <c r="B36" s="120" t="s">
+    <row r="36" spans="1:20">
+      <c r="A36" s="103"/>
+      <c r="B36" s="108" t="s">
         <v>393</v>
       </c>
-      <c r="C36" s="120" t="s">
+      <c r="C36" s="108" t="s">
         <v>394</v>
       </c>
-      <c r="D36" s="120" t="s">
+      <c r="D36" s="108" t="s">
         <v>395</v>
       </c>
-      <c r="E36" s="120" t="s">
+      <c r="E36" s="108" t="s">
         <v>396</v>
       </c>
-      <c r="F36" s="120" t="s">
+      <c r="F36" s="108" t="s">
         <v>397</v>
       </c>
       <c r="G36" s="35" t="s">
@@ -7861,7 +7861,7 @@
       <c r="H36" s="35" t="s">
         <v>399</v>
       </c>
-      <c r="I36" s="120" t="s">
+      <c r="I36" s="108" t="s">
         <v>362</v>
       </c>
       <c r="J36" s="35" t="s">
@@ -7870,56 +7870,56 @@
       <c r="K36" s="40" t="s">
         <v>392</v>
       </c>
-      <c r="L36" s="121"/>
+      <c r="L36" s="109"/>
       <c r="M36" s="38"/>
     </row>
     <row r="37" spans="1:20">
-      <c r="A37" s="116"/>
-      <c r="B37" s="122"/>
-      <c r="C37" s="122"/>
-      <c r="D37" s="122"/>
-      <c r="E37" s="122"/>
-      <c r="F37" s="122"/>
+      <c r="A37" s="104"/>
+      <c r="B37" s="110"/>
+      <c r="C37" s="110"/>
+      <c r="D37" s="110"/>
+      <c r="E37" s="110"/>
+      <c r="F37" s="110"/>
       <c r="G37" s="42" t="s">
         <v>392</v>
       </c>
       <c r="H37" s="43" t="s">
         <v>399</v>
       </c>
-      <c r="I37" s="122"/>
+      <c r="I37" s="110"/>
       <c r="J37" s="42" t="s">
         <v>392</v>
       </c>
       <c r="K37" s="41"/>
-      <c r="L37" s="122"/>
+      <c r="L37" s="110"/>
       <c r="M37" s="39"/>
     </row>
     <row r="38" spans="1:20">
-      <c r="A38" s="125">
+      <c r="A38" s="100">
         <v>2024</v>
       </c>
-      <c r="B38" s="123">
+      <c r="B38" s="96">
         <v>34160</v>
       </c>
-      <c r="C38" s="123">
+      <c r="C38" s="96">
         <v>4330</v>
       </c>
-      <c r="D38" s="123">
+      <c r="D38" s="96">
         <v>3633</v>
       </c>
-      <c r="E38" s="127">
+      <c r="E38" s="98">
         <v>446</v>
       </c>
-      <c r="F38" s="123">
+      <c r="F38" s="96">
         <v>11146</v>
       </c>
       <c r="G38" s="45">
         <v>53716</v>
       </c>
-      <c r="H38" s="123">
+      <c r="H38" s="96">
         <v>7277</v>
       </c>
-      <c r="I38" s="123">
+      <c r="I38" s="96">
         <v>2182</v>
       </c>
       <c r="J38" s="45">
@@ -7928,7 +7928,7 @@
       <c r="K38" s="45">
         <v>63174</v>
       </c>
-      <c r="L38" s="123">
+      <c r="L38" s="96">
         <v>5956</v>
       </c>
       <c r="M38" s="47">
@@ -7937,55 +7937,55 @@
       <c r="N38" s="51"/>
     </row>
     <row r="39" spans="1:20">
-      <c r="A39" s="126"/>
-      <c r="B39" s="124"/>
-      <c r="C39" s="124"/>
-      <c r="D39" s="124"/>
-      <c r="E39" s="128"/>
-      <c r="F39" s="124"/>
+      <c r="A39" s="101"/>
+      <c r="B39" s="97"/>
+      <c r="C39" s="97"/>
+      <c r="D39" s="97"/>
+      <c r="E39" s="99"/>
+      <c r="F39" s="97"/>
       <c r="G39" s="46">
         <v>9</v>
       </c>
-      <c r="H39" s="124"/>
-      <c r="I39" s="124"/>
+      <c r="H39" s="97"/>
+      <c r="I39" s="97"/>
       <c r="J39" s="46">
         <v>1.6</v>
       </c>
       <c r="K39" s="46">
         <v>10.5</v>
       </c>
-      <c r="L39" s="124"/>
+      <c r="L39" s="97"/>
       <c r="M39" s="48">
         <v>10.8</v>
       </c>
       <c r="N39" s="51"/>
     </row>
     <row r="40" spans="1:20">
-      <c r="A40" s="125">
+      <c r="A40" s="100">
         <v>2025</v>
       </c>
-      <c r="B40" s="123">
+      <c r="B40" s="96">
         <v>39140</v>
       </c>
-      <c r="C40" s="123">
+      <c r="C40" s="96">
         <v>5255</v>
       </c>
-      <c r="D40" s="123">
+      <c r="D40" s="96">
         <v>3712</v>
       </c>
-      <c r="E40" s="127">
+      <c r="E40" s="98">
         <v>445</v>
       </c>
-      <c r="F40" s="123">
+      <c r="F40" s="96">
         <v>11164</v>
       </c>
       <c r="G40" s="45">
         <v>59716</v>
       </c>
-      <c r="H40" s="123">
+      <c r="H40" s="96">
         <v>8832</v>
       </c>
-      <c r="I40" s="123">
+      <c r="I40" s="96">
         <v>2176</v>
       </c>
       <c r="J40" s="45">
@@ -7994,7 +7994,7 @@
       <c r="K40" s="45">
         <v>70723</v>
       </c>
-      <c r="L40" s="123">
+      <c r="L40" s="96">
         <v>6549</v>
       </c>
       <c r="M40" s="47">
@@ -8009,24 +8009,24 @@
       <c r="T40" s="51"/>
     </row>
     <row r="41" spans="1:20">
-      <c r="A41" s="126"/>
-      <c r="B41" s="124"/>
-      <c r="C41" s="124"/>
-      <c r="D41" s="124"/>
-      <c r="E41" s="128"/>
-      <c r="F41" s="124"/>
+      <c r="A41" s="101"/>
+      <c r="B41" s="97"/>
+      <c r="C41" s="97"/>
+      <c r="D41" s="97"/>
+      <c r="E41" s="99"/>
+      <c r="F41" s="97"/>
       <c r="G41" s="46">
         <v>9.8000000000000007</v>
       </c>
-      <c r="H41" s="124"/>
-      <c r="I41" s="124"/>
+      <c r="H41" s="97"/>
+      <c r="I41" s="97"/>
       <c r="J41" s="46">
         <v>1.8</v>
       </c>
       <c r="K41" s="46">
         <v>11.7</v>
       </c>
-      <c r="L41" s="124"/>
+      <c r="L41" s="97"/>
       <c r="M41" s="48">
         <v>11.9</v>
       </c>
@@ -8039,31 +8039,31 @@
       <c r="T41" s="51"/>
     </row>
     <row r="42" spans="1:20">
-      <c r="A42" s="125">
+      <c r="A42" s="100">
         <v>2026</v>
       </c>
-      <c r="B42" s="123">
+      <c r="B42" s="96">
         <v>44154</v>
       </c>
-      <c r="C42" s="123">
+      <c r="C42" s="96">
         <v>6889</v>
       </c>
-      <c r="D42" s="123">
+      <c r="D42" s="96">
         <v>3712</v>
       </c>
-      <c r="E42" s="127">
+      <c r="E42" s="98">
         <v>445</v>
       </c>
-      <c r="F42" s="123">
+      <c r="F42" s="96">
         <v>10870</v>
       </c>
       <c r="G42" s="45">
         <v>66070</v>
       </c>
-      <c r="H42" s="123">
+      <c r="H42" s="96">
         <v>10631</v>
       </c>
-      <c r="I42" s="123">
+      <c r="I42" s="96">
         <v>2176</v>
       </c>
       <c r="J42" s="45">
@@ -8072,7 +8072,7 @@
       <c r="K42" s="45">
         <v>78877</v>
       </c>
-      <c r="L42" s="123">
+      <c r="L42" s="96">
         <v>7212</v>
       </c>
       <c r="M42" s="47">
@@ -8087,24 +8087,24 @@
       <c r="T42" s="51"/>
     </row>
     <row r="43" spans="1:20">
-      <c r="A43" s="126"/>
-      <c r="B43" s="124"/>
-      <c r="C43" s="124"/>
-      <c r="D43" s="124"/>
-      <c r="E43" s="128"/>
-      <c r="F43" s="124"/>
+      <c r="A43" s="101"/>
+      <c r="B43" s="97"/>
+      <c r="C43" s="97"/>
+      <c r="D43" s="97"/>
+      <c r="E43" s="99"/>
+      <c r="F43" s="97"/>
       <c r="G43" s="46">
         <v>10.8</v>
       </c>
-      <c r="H43" s="124"/>
-      <c r="I43" s="124"/>
+      <c r="H43" s="97"/>
+      <c r="I43" s="97"/>
       <c r="J43" s="46">
         <v>2.1</v>
       </c>
       <c r="K43" s="46">
         <v>12.8</v>
       </c>
-      <c r="L43" s="124"/>
+      <c r="L43" s="97"/>
       <c r="M43" s="48">
         <v>13.1</v>
       </c>
@@ -8117,31 +8117,31 @@
       <c r="T43" s="51"/>
     </row>
     <row r="44" spans="1:20">
-      <c r="A44" s="125">
+      <c r="A44" s="100">
         <v>2027</v>
       </c>
-      <c r="B44" s="123">
+      <c r="B44" s="96">
         <v>49055</v>
       </c>
-      <c r="C44" s="123">
+      <c r="C44" s="96">
         <v>10369</v>
       </c>
-      <c r="D44" s="123">
+      <c r="D44" s="96">
         <v>3712</v>
       </c>
-      <c r="E44" s="127">
+      <c r="E44" s="98">
         <v>445</v>
       </c>
-      <c r="F44" s="123">
+      <c r="F44" s="96">
         <v>10863</v>
       </c>
       <c r="G44" s="45">
         <v>74445</v>
       </c>
-      <c r="H44" s="123">
+      <c r="H44" s="96">
         <v>12179</v>
       </c>
-      <c r="I44" s="123">
+      <c r="I44" s="96">
         <v>2176</v>
       </c>
       <c r="J44" s="45">
@@ -8150,7 +8150,7 @@
       <c r="K44" s="45">
         <v>88799</v>
       </c>
-      <c r="L44" s="123">
+      <c r="L44" s="96">
         <v>7896</v>
       </c>
       <c r="M44" s="47">
@@ -8165,24 +8165,24 @@
       <c r="T44" s="51"/>
     </row>
     <row r="45" spans="1:20">
-      <c r="A45" s="126"/>
-      <c r="B45" s="124"/>
-      <c r="C45" s="124"/>
-      <c r="D45" s="124"/>
-      <c r="E45" s="128"/>
-      <c r="F45" s="124"/>
+      <c r="A45" s="101"/>
+      <c r="B45" s="97"/>
+      <c r="C45" s="97"/>
+      <c r="D45" s="97"/>
+      <c r="E45" s="99"/>
+      <c r="F45" s="97"/>
       <c r="G45" s="46">
         <v>12</v>
       </c>
-      <c r="H45" s="124"/>
-      <c r="I45" s="124"/>
+      <c r="H45" s="97"/>
+      <c r="I45" s="97"/>
       <c r="J45" s="46">
         <v>2.2999999999999998</v>
       </c>
       <c r="K45" s="46">
         <v>14.3</v>
       </c>
-      <c r="L45" s="124"/>
+      <c r="L45" s="97"/>
       <c r="M45" s="48">
         <v>14.5</v>
       </c>
@@ -8207,19 +8207,19 @@
       <c r="D46" s="45">
         <v>3722</v>
       </c>
-      <c r="E46" s="127">
+      <c r="E46" s="98">
         <v>446</v>
       </c>
-      <c r="F46" s="123">
+      <c r="F46" s="96">
         <v>10878</v>
       </c>
       <c r="G46" s="45">
         <v>86001</v>
       </c>
-      <c r="H46" s="123">
+      <c r="H46" s="96">
         <v>13656</v>
       </c>
-      <c r="I46" s="123">
+      <c r="I46" s="96">
         <v>2182</v>
       </c>
       <c r="J46" s="45">
@@ -8228,7 +8228,7 @@
       <c r="K46" s="45">
         <v>101839</v>
       </c>
-      <c r="L46" s="123">
+      <c r="L46" s="96">
         <v>8626</v>
       </c>
       <c r="M46" s="47">
@@ -8247,20 +8247,20 @@
       <c r="B47" s="50"/>
       <c r="C47" s="50"/>
       <c r="D47" s="50"/>
-      <c r="E47" s="128"/>
-      <c r="F47" s="124"/>
+      <c r="E47" s="99"/>
+      <c r="F47" s="97"/>
       <c r="G47" s="46">
         <v>13.7</v>
       </c>
-      <c r="H47" s="124"/>
-      <c r="I47" s="124"/>
+      <c r="H47" s="97"/>
+      <c r="I47" s="97"/>
       <c r="J47" s="46">
         <v>2.5</v>
       </c>
       <c r="K47" s="46">
         <v>16.2</v>
       </c>
-      <c r="L47" s="124"/>
+      <c r="L47" s="97"/>
       <c r="M47" s="48">
         <v>16.3</v>
       </c>
@@ -8285,19 +8285,19 @@
       <c r="D48" s="45">
         <v>3712</v>
       </c>
-      <c r="E48" s="127">
+      <c r="E48" s="98">
         <v>445</v>
       </c>
-      <c r="F48" s="123">
+      <c r="F48" s="96">
         <v>10846</v>
       </c>
       <c r="G48" s="45">
         <v>102096</v>
       </c>
-      <c r="H48" s="123">
+      <c r="H48" s="96">
         <v>15059</v>
       </c>
-      <c r="I48" s="123">
+      <c r="I48" s="96">
         <v>2176</v>
       </c>
       <c r="J48" s="45">
@@ -8306,7 +8306,7 @@
       <c r="K48" s="45">
         <v>119331</v>
       </c>
-      <c r="L48" s="123">
+      <c r="L48" s="96">
         <v>9328</v>
       </c>
       <c r="M48" s="47">
@@ -8325,20 +8325,20 @@
       <c r="B49" s="50"/>
       <c r="C49" s="50"/>
       <c r="D49" s="50"/>
-      <c r="E49" s="128"/>
-      <c r="F49" s="124"/>
+      <c r="E49" s="99"/>
+      <c r="F49" s="97"/>
       <c r="G49" s="46">
         <v>16.100000000000001</v>
       </c>
-      <c r="H49" s="124"/>
-      <c r="I49" s="124"/>
+      <c r="H49" s="97"/>
+      <c r="I49" s="97"/>
       <c r="J49" s="46">
         <v>2.7</v>
       </c>
       <c r="K49" s="46">
         <v>18.8</v>
       </c>
-      <c r="L49" s="124"/>
+      <c r="L49" s="97"/>
       <c r="M49" s="48">
         <v>18.899999999999999</v>
       </c>
@@ -8363,19 +8363,19 @@
       <c r="D50" s="45">
         <v>3712</v>
       </c>
-      <c r="E50" s="127">
+      <c r="E50" s="98">
         <v>445</v>
       </c>
-      <c r="F50" s="123">
+      <c r="F50" s="96">
         <v>10814</v>
       </c>
       <c r="G50" s="45">
         <v>120920</v>
       </c>
-      <c r="H50" s="123">
+      <c r="H50" s="96">
         <v>16500</v>
       </c>
-      <c r="I50" s="123">
+      <c r="I50" s="96">
         <v>2176</v>
       </c>
       <c r="J50" s="45">
@@ -8384,7 +8384,7 @@
       <c r="K50" s="45">
         <v>139595</v>
       </c>
-      <c r="L50" s="123">
+      <c r="L50" s="96">
         <v>10071</v>
       </c>
       <c r="M50" s="47">
@@ -8403,20 +8403,20 @@
       <c r="B51" s="50"/>
       <c r="C51" s="50"/>
       <c r="D51" s="50"/>
-      <c r="E51" s="128"/>
-      <c r="F51" s="124"/>
+      <c r="E51" s="99"/>
+      <c r="F51" s="97"/>
       <c r="G51" s="46">
         <v>18.8</v>
       </c>
-      <c r="H51" s="124"/>
-      <c r="I51" s="124"/>
+      <c r="H51" s="97"/>
+      <c r="I51" s="97"/>
       <c r="J51" s="46">
         <v>2.9</v>
       </c>
       <c r="K51" s="46">
         <v>21.7</v>
       </c>
-      <c r="L51" s="124"/>
+      <c r="L51" s="97"/>
       <c r="M51" s="48">
         <v>21.7</v>
       </c>
@@ -8441,19 +8441,19 @@
       <c r="D52" s="45">
         <v>3712</v>
       </c>
-      <c r="E52" s="127">
+      <c r="E52" s="98">
         <v>445</v>
       </c>
-      <c r="F52" s="123">
+      <c r="F52" s="96">
         <v>10815</v>
       </c>
       <c r="G52" s="45">
         <v>136599</v>
       </c>
-      <c r="H52" s="123">
+      <c r="H52" s="96">
         <v>17760</v>
       </c>
-      <c r="I52" s="123">
+      <c r="I52" s="96">
         <v>2176</v>
       </c>
       <c r="J52" s="45">
@@ -8462,7 +8462,7 @@
       <c r="K52" s="45">
         <v>156535</v>
       </c>
-      <c r="L52" s="123">
+      <c r="L52" s="96">
         <v>10824</v>
       </c>
       <c r="M52" s="47">
@@ -8481,20 +8481,20 @@
       <c r="B53" s="50"/>
       <c r="C53" s="50"/>
       <c r="D53" s="50"/>
-      <c r="E53" s="128"/>
-      <c r="F53" s="124"/>
+      <c r="E53" s="99"/>
+      <c r="F53" s="97"/>
       <c r="G53" s="46">
         <v>20.9</v>
       </c>
-      <c r="H53" s="124"/>
-      <c r="I53" s="124"/>
+      <c r="H53" s="97"/>
+      <c r="I53" s="97"/>
       <c r="J53" s="46">
         <v>3</v>
       </c>
       <c r="K53" s="46">
         <v>23.9</v>
       </c>
-      <c r="L53" s="124"/>
+      <c r="L53" s="97"/>
       <c r="M53" s="48">
         <v>23.8</v>
       </c>
@@ -8519,19 +8519,19 @@
       <c r="D54" s="45">
         <v>3722</v>
       </c>
-      <c r="E54" s="127">
+      <c r="E54" s="98">
         <v>446</v>
       </c>
-      <c r="F54" s="123">
+      <c r="F54" s="96">
         <v>10845</v>
       </c>
       <c r="G54" s="45">
         <v>149056</v>
       </c>
-      <c r="H54" s="123">
+      <c r="H54" s="96">
         <v>18892</v>
       </c>
-      <c r="I54" s="123">
+      <c r="I54" s="96">
         <v>2182</v>
       </c>
       <c r="J54" s="45">
@@ -8540,7 +8540,7 @@
       <c r="K54" s="45">
         <v>170130</v>
       </c>
-      <c r="L54" s="123">
+      <c r="L54" s="96">
         <v>11617</v>
       </c>
       <c r="M54" s="47">
@@ -8559,20 +8559,20 @@
       <c r="B55" s="50"/>
       <c r="C55" s="50"/>
       <c r="D55" s="50"/>
-      <c r="E55" s="128"/>
-      <c r="F55" s="124"/>
+      <c r="E55" s="99"/>
+      <c r="F55" s="97"/>
       <c r="G55" s="46">
         <v>22.4</v>
       </c>
-      <c r="H55" s="124"/>
-      <c r="I55" s="124"/>
+      <c r="H55" s="97"/>
+      <c r="I55" s="97"/>
       <c r="J55" s="46">
         <v>3.2</v>
       </c>
       <c r="K55" s="46">
         <v>25.6</v>
       </c>
-      <c r="L55" s="124"/>
+      <c r="L55" s="97"/>
       <c r="M55" s="48">
         <v>25.4</v>
       </c>
@@ -8597,19 +8597,19 @@
       <c r="D56" s="45">
         <v>3712</v>
       </c>
-      <c r="E56" s="127">
+      <c r="E56" s="98">
         <v>445</v>
       </c>
-      <c r="F56" s="123">
+      <c r="F56" s="96">
         <v>10803</v>
       </c>
       <c r="G56" s="45">
         <v>158886</v>
       </c>
-      <c r="H56" s="123">
+      <c r="H56" s="96">
         <v>19920</v>
       </c>
-      <c r="I56" s="123">
+      <c r="I56" s="96">
         <v>2176</v>
       </c>
       <c r="J56" s="45">
@@ -8618,7 +8618,7 @@
       <c r="K56" s="45">
         <v>180982</v>
       </c>
-      <c r="L56" s="123">
+      <c r="L56" s="96">
         <v>12363</v>
       </c>
       <c r="M56" s="47">
@@ -8637,20 +8637,20 @@
       <c r="B57" s="50"/>
       <c r="C57" s="50"/>
       <c r="D57" s="50"/>
-      <c r="E57" s="128"/>
-      <c r="F57" s="124"/>
+      <c r="E57" s="99"/>
+      <c r="F57" s="97"/>
       <c r="G57" s="46">
         <v>23.6</v>
       </c>
-      <c r="H57" s="124"/>
-      <c r="I57" s="124"/>
+      <c r="H57" s="97"/>
+      <c r="I57" s="97"/>
       <c r="J57" s="46">
         <v>3.3</v>
       </c>
       <c r="K57" s="46">
         <v>26.9</v>
       </c>
-      <c r="L57" s="124"/>
+      <c r="L57" s="97"/>
       <c r="M57" s="48">
         <v>26.7</v>
       </c>
@@ -8675,19 +8675,19 @@
       <c r="D58" s="45">
         <v>3712</v>
       </c>
-      <c r="E58" s="127">
+      <c r="E58" s="98">
         <v>445</v>
       </c>
-      <c r="F58" s="123">
+      <c r="F58" s="96">
         <v>10817</v>
       </c>
       <c r="G58" s="45">
         <v>169108</v>
       </c>
-      <c r="H58" s="123">
+      <c r="H58" s="96">
         <v>21000</v>
       </c>
-      <c r="I58" s="123">
+      <c r="I58" s="96">
         <v>2176</v>
       </c>
       <c r="J58" s="45">
@@ -8696,7 +8696,7 @@
       <c r="K58" s="45">
         <v>192284</v>
       </c>
-      <c r="L58" s="123">
+      <c r="L58" s="96">
         <v>13159</v>
       </c>
       <c r="M58" s="47">
@@ -8715,20 +8715,20 @@
       <c r="B59" s="50"/>
       <c r="C59" s="50"/>
       <c r="D59" s="50"/>
-      <c r="E59" s="128"/>
-      <c r="F59" s="124"/>
+      <c r="E59" s="99"/>
+      <c r="F59" s="97"/>
       <c r="G59" s="46">
         <v>24.8</v>
       </c>
-      <c r="H59" s="124"/>
-      <c r="I59" s="124"/>
+      <c r="H59" s="97"/>
+      <c r="I59" s="97"/>
       <c r="J59" s="46">
         <v>3.4</v>
       </c>
       <c r="K59" s="46">
         <v>28.2</v>
       </c>
-      <c r="L59" s="124"/>
+      <c r="L59" s="97"/>
       <c r="M59" s="48">
         <v>28</v>
       </c>
@@ -8753,19 +8753,19 @@
       <c r="D60" s="45">
         <v>3712</v>
       </c>
-      <c r="E60" s="127">
+      <c r="E60" s="98">
         <v>445</v>
       </c>
-      <c r="F60" s="123">
+      <c r="F60" s="96">
         <v>10799</v>
       </c>
       <c r="G60" s="45">
         <v>179937</v>
       </c>
-      <c r="H60" s="123">
+      <c r="H60" s="96">
         <v>22081</v>
       </c>
-      <c r="I60" s="123">
+      <c r="I60" s="96">
         <v>2176</v>
       </c>
       <c r="J60" s="45">
@@ -8774,7 +8774,7 @@
       <c r="K60" s="45">
         <v>204193</v>
       </c>
-      <c r="L60" s="123">
+      <c r="L60" s="96">
         <v>13973</v>
       </c>
       <c r="M60" s="47">
@@ -8793,20 +8793,20 @@
       <c r="B61" s="50"/>
       <c r="C61" s="50"/>
       <c r="D61" s="50"/>
-      <c r="E61" s="128"/>
-      <c r="F61" s="124"/>
+      <c r="E61" s="99"/>
+      <c r="F61" s="97"/>
       <c r="G61" s="46">
         <v>26</v>
       </c>
-      <c r="H61" s="124"/>
-      <c r="I61" s="124"/>
+      <c r="H61" s="97"/>
+      <c r="I61" s="97"/>
       <c r="J61" s="46">
         <v>3.5</v>
       </c>
       <c r="K61" s="46">
         <v>29.5</v>
       </c>
-      <c r="L61" s="124"/>
+      <c r="L61" s="97"/>
       <c r="M61" s="48">
         <v>29.3</v>
       </c>
@@ -8831,19 +8831,19 @@
       <c r="D62" s="45">
         <v>3722</v>
       </c>
-      <c r="E62" s="127">
+      <c r="E62" s="98">
         <v>446</v>
       </c>
-      <c r="F62" s="123">
+      <c r="F62" s="96">
         <v>10633</v>
       </c>
       <c r="G62" s="45">
         <v>190398</v>
       </c>
-      <c r="H62" s="123">
+      <c r="H62" s="96">
         <v>22745</v>
       </c>
-      <c r="I62" s="123">
+      <c r="I62" s="96">
         <v>2182</v>
       </c>
       <c r="J62" s="45">
@@ -8852,7 +8852,7 @@
       <c r="K62" s="45">
         <v>215325</v>
       </c>
-      <c r="L62" s="123">
+      <c r="L62" s="96">
         <v>14845</v>
       </c>
       <c r="M62" s="47">
@@ -8871,20 +8871,20 @@
       <c r="B63" s="50"/>
       <c r="C63" s="50"/>
       <c r="D63" s="50"/>
-      <c r="E63" s="128"/>
-      <c r="F63" s="124"/>
+      <c r="E63" s="99"/>
+      <c r="F63" s="97"/>
       <c r="G63" s="46">
         <v>27.5</v>
       </c>
-      <c r="H63" s="124"/>
-      <c r="I63" s="124"/>
+      <c r="H63" s="97"/>
+      <c r="I63" s="97"/>
       <c r="J63" s="46">
         <v>3.6</v>
       </c>
       <c r="K63" s="46">
         <v>31.1</v>
       </c>
-      <c r="L63" s="124"/>
+      <c r="L63" s="97"/>
       <c r="M63" s="48">
         <v>30.8</v>
       </c>
@@ -8909,19 +8909,19 @@
       <c r="D64" s="45">
         <v>3712</v>
       </c>
-      <c r="E64" s="127">
+      <c r="E64" s="98">
         <v>445</v>
       </c>
-      <c r="F64" s="123">
+      <c r="F64" s="96">
         <v>10600</v>
       </c>
       <c r="G64" s="45">
         <v>198295</v>
       </c>
-      <c r="H64" s="123">
+      <c r="H64" s="96">
         <v>23565</v>
       </c>
-      <c r="I64" s="123">
+      <c r="I64" s="96">
         <v>2176</v>
       </c>
       <c r="J64" s="45">
@@ -8930,7 +8930,7 @@
       <c r="K64" s="45">
         <v>224035</v>
       </c>
-      <c r="L64" s="123">
+      <c r="L64" s="96">
         <v>15655</v>
       </c>
       <c r="M64" s="47">
@@ -8949,20 +8949,20 @@
       <c r="B65" s="50"/>
       <c r="C65" s="50"/>
       <c r="D65" s="50"/>
-      <c r="E65" s="128"/>
-      <c r="F65" s="124"/>
+      <c r="E65" s="99"/>
+      <c r="F65" s="97"/>
       <c r="G65" s="46">
         <v>28.4</v>
       </c>
-      <c r="H65" s="124"/>
-      <c r="I65" s="124"/>
+      <c r="H65" s="97"/>
+      <c r="I65" s="97"/>
       <c r="J65" s="46">
         <v>3.7</v>
       </c>
       <c r="K65" s="46">
         <v>32.1</v>
       </c>
-      <c r="L65" s="124"/>
+      <c r="L65" s="97"/>
       <c r="M65" s="48">
         <v>31.9</v>
       </c>
@@ -8987,19 +8987,19 @@
       <c r="D66" s="45">
         <v>3712</v>
       </c>
-      <c r="E66" s="127">
+      <c r="E66" s="98">
         <v>445</v>
       </c>
-      <c r="F66" s="123">
+      <c r="F66" s="96">
         <v>10602</v>
       </c>
       <c r="G66" s="45">
         <v>205673</v>
       </c>
-      <c r="H66" s="123">
+      <c r="H66" s="96">
         <v>24270</v>
       </c>
-      <c r="I66" s="123">
+      <c r="I66" s="96">
         <v>2176</v>
       </c>
       <c r="J66" s="45">
@@ -9008,7 +9008,7 @@
       <c r="K66" s="45">
         <v>232119</v>
       </c>
-      <c r="L66" s="123">
+      <c r="L66" s="96">
         <v>16523</v>
       </c>
       <c r="M66" s="47">
@@ -9027,20 +9027,20 @@
       <c r="B67" s="50"/>
       <c r="C67" s="50"/>
       <c r="D67" s="50"/>
-      <c r="E67" s="128"/>
-      <c r="F67" s="124"/>
+      <c r="E67" s="99"/>
+      <c r="F67" s="97"/>
       <c r="G67" s="46">
         <v>29.2</v>
       </c>
-      <c r="H67" s="124"/>
-      <c r="I67" s="124"/>
+      <c r="H67" s="97"/>
+      <c r="I67" s="97"/>
       <c r="J67" s="46">
         <v>3.8</v>
       </c>
       <c r="K67" s="46">
         <v>32.9</v>
       </c>
-      <c r="L67" s="124"/>
+      <c r="L67" s="97"/>
       <c r="M67" s="48">
         <v>32.700000000000003</v>
       </c>
@@ -9350,61 +9350,59 @@
     </row>
   </sheetData>
   <mergeCells count="126">
-    <mergeCell ref="F66:F67"/>
-    <mergeCell ref="H66:H67"/>
-    <mergeCell ref="I66:I67"/>
-    <mergeCell ref="L66:L67"/>
-    <mergeCell ref="E66:E67"/>
-    <mergeCell ref="F62:F63"/>
-    <mergeCell ref="H62:H63"/>
-    <mergeCell ref="I62:I63"/>
-    <mergeCell ref="L62:L63"/>
-    <mergeCell ref="E64:E65"/>
-    <mergeCell ref="F64:F65"/>
-    <mergeCell ref="H64:H65"/>
-    <mergeCell ref="I64:I65"/>
-    <mergeCell ref="L64:L65"/>
-    <mergeCell ref="E62:E63"/>
-    <mergeCell ref="F58:F59"/>
-    <mergeCell ref="H58:H59"/>
-    <mergeCell ref="I58:I59"/>
-    <mergeCell ref="L58:L59"/>
-    <mergeCell ref="E60:E61"/>
-    <mergeCell ref="F60:F61"/>
-    <mergeCell ref="H60:H61"/>
-    <mergeCell ref="I60:I61"/>
-    <mergeCell ref="L60:L61"/>
-    <mergeCell ref="E58:E59"/>
-    <mergeCell ref="F54:F55"/>
-    <mergeCell ref="H54:H55"/>
-    <mergeCell ref="I54:I55"/>
-    <mergeCell ref="L54:L55"/>
-    <mergeCell ref="E56:E57"/>
-    <mergeCell ref="F56:F57"/>
-    <mergeCell ref="H56:H57"/>
-    <mergeCell ref="I56:I57"/>
-    <mergeCell ref="L56:L57"/>
-    <mergeCell ref="E54:E55"/>
-    <mergeCell ref="F50:F51"/>
-    <mergeCell ref="H50:H51"/>
-    <mergeCell ref="I50:I51"/>
-    <mergeCell ref="L50:L51"/>
-    <mergeCell ref="E52:E53"/>
-    <mergeCell ref="F52:F53"/>
-    <mergeCell ref="H52:H53"/>
-    <mergeCell ref="I52:I53"/>
-    <mergeCell ref="L52:L53"/>
-    <mergeCell ref="E50:E51"/>
-    <mergeCell ref="F46:F47"/>
-    <mergeCell ref="H46:H47"/>
-    <mergeCell ref="I46:I47"/>
-    <mergeCell ref="L46:L47"/>
-    <mergeCell ref="E48:E49"/>
-    <mergeCell ref="F48:F49"/>
-    <mergeCell ref="H48:H49"/>
-    <mergeCell ref="I48:I49"/>
-    <mergeCell ref="L48:L49"/>
-    <mergeCell ref="E46:E47"/>
+    <mergeCell ref="B1:F1"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="K23:L23"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="D21:D22"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="G21:G22"/>
+    <mergeCell ref="H21:H22"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="L21:M21"/>
+    <mergeCell ref="K22:L22"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="K29:L29"/>
+    <mergeCell ref="K30:L30"/>
+    <mergeCell ref="K24:L24"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="K25:L25"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="K27:L27"/>
+    <mergeCell ref="K28:L28"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="B34:K34"/>
+    <mergeCell ref="L34:L37"/>
+    <mergeCell ref="B35:G35"/>
+    <mergeCell ref="H35:J35"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="C36:C37"/>
+    <mergeCell ref="D36:D37"/>
+    <mergeCell ref="E36:E37"/>
+    <mergeCell ref="F36:F37"/>
+    <mergeCell ref="I36:I37"/>
+    <mergeCell ref="F38:F39"/>
+    <mergeCell ref="H38:H39"/>
+    <mergeCell ref="I38:I39"/>
+    <mergeCell ref="L38:L39"/>
+    <mergeCell ref="A40:A41"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="C40:C41"/>
+    <mergeCell ref="D40:D41"/>
+    <mergeCell ref="E40:E41"/>
+    <mergeCell ref="F40:F41"/>
+    <mergeCell ref="H40:H41"/>
+    <mergeCell ref="I40:I41"/>
+    <mergeCell ref="L40:L41"/>
+    <mergeCell ref="A38:A39"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="D38:D39"/>
+    <mergeCell ref="E38:E39"/>
     <mergeCell ref="F42:F43"/>
     <mergeCell ref="H42:H43"/>
     <mergeCell ref="I42:I43"/>
@@ -9423,59 +9421,61 @@
     <mergeCell ref="C42:C43"/>
     <mergeCell ref="D42:D43"/>
     <mergeCell ref="E42:E43"/>
-    <mergeCell ref="F38:F39"/>
-    <mergeCell ref="H38:H39"/>
-    <mergeCell ref="I38:I39"/>
-    <mergeCell ref="L38:L39"/>
-    <mergeCell ref="A40:A41"/>
-    <mergeCell ref="B40:B41"/>
-    <mergeCell ref="C40:C41"/>
-    <mergeCell ref="D40:D41"/>
-    <mergeCell ref="E40:E41"/>
-    <mergeCell ref="F40:F41"/>
-    <mergeCell ref="H40:H41"/>
-    <mergeCell ref="I40:I41"/>
-    <mergeCell ref="L40:L41"/>
-    <mergeCell ref="A38:A39"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="C38:C39"/>
-    <mergeCell ref="D38:D39"/>
-    <mergeCell ref="E38:E39"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="B34:K34"/>
-    <mergeCell ref="L34:L37"/>
-    <mergeCell ref="B35:G35"/>
-    <mergeCell ref="H35:J35"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="C36:C37"/>
-    <mergeCell ref="D36:D37"/>
-    <mergeCell ref="E36:E37"/>
-    <mergeCell ref="F36:F37"/>
-    <mergeCell ref="I36:I37"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="K29:L29"/>
-    <mergeCell ref="K30:L30"/>
-    <mergeCell ref="K24:L24"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="K25:L25"/>
-    <mergeCell ref="K26:L26"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="K27:L27"/>
-    <mergeCell ref="K28:L28"/>
-    <mergeCell ref="B1:F1"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="K23:L23"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="D21:D22"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="F21:F22"/>
-    <mergeCell ref="G21:G22"/>
-    <mergeCell ref="H21:H22"/>
-    <mergeCell ref="I21:I22"/>
-    <mergeCell ref="J21:J22"/>
-    <mergeCell ref="L21:M21"/>
-    <mergeCell ref="K22:L22"/>
+    <mergeCell ref="F46:F47"/>
+    <mergeCell ref="H46:H47"/>
+    <mergeCell ref="I46:I47"/>
+    <mergeCell ref="L46:L47"/>
+    <mergeCell ref="E48:E49"/>
+    <mergeCell ref="F48:F49"/>
+    <mergeCell ref="H48:H49"/>
+    <mergeCell ref="I48:I49"/>
+    <mergeCell ref="L48:L49"/>
+    <mergeCell ref="E46:E47"/>
+    <mergeCell ref="F50:F51"/>
+    <mergeCell ref="H50:H51"/>
+    <mergeCell ref="I50:I51"/>
+    <mergeCell ref="L50:L51"/>
+    <mergeCell ref="E52:E53"/>
+    <mergeCell ref="F52:F53"/>
+    <mergeCell ref="H52:H53"/>
+    <mergeCell ref="I52:I53"/>
+    <mergeCell ref="L52:L53"/>
+    <mergeCell ref="E50:E51"/>
+    <mergeCell ref="F54:F55"/>
+    <mergeCell ref="H54:H55"/>
+    <mergeCell ref="I54:I55"/>
+    <mergeCell ref="L54:L55"/>
+    <mergeCell ref="E56:E57"/>
+    <mergeCell ref="F56:F57"/>
+    <mergeCell ref="H56:H57"/>
+    <mergeCell ref="I56:I57"/>
+    <mergeCell ref="L56:L57"/>
+    <mergeCell ref="E54:E55"/>
+    <mergeCell ref="F58:F59"/>
+    <mergeCell ref="H58:H59"/>
+    <mergeCell ref="I58:I59"/>
+    <mergeCell ref="L58:L59"/>
+    <mergeCell ref="E60:E61"/>
+    <mergeCell ref="F60:F61"/>
+    <mergeCell ref="H60:H61"/>
+    <mergeCell ref="I60:I61"/>
+    <mergeCell ref="L60:L61"/>
+    <mergeCell ref="E58:E59"/>
+    <mergeCell ref="F66:F67"/>
+    <mergeCell ref="H66:H67"/>
+    <mergeCell ref="I66:I67"/>
+    <mergeCell ref="L66:L67"/>
+    <mergeCell ref="E66:E67"/>
+    <mergeCell ref="F62:F63"/>
+    <mergeCell ref="H62:H63"/>
+    <mergeCell ref="I62:I63"/>
+    <mergeCell ref="L62:L63"/>
+    <mergeCell ref="E64:E65"/>
+    <mergeCell ref="F64:F65"/>
+    <mergeCell ref="H64:H65"/>
+    <mergeCell ref="I64:I65"/>
+    <mergeCell ref="L64:L65"/>
+    <mergeCell ref="E62:E63"/>
   </mergeCells>
   <phoneticPr fontId="26" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9486,9 +9486,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72E1B7E2-B244-47F8-B566-550E2814D46F}">
   <dimension ref="A1:CC20"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="70.7109375" customWidth="1"/>
+    <col min="1" max="1" width="70.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:81">
@@ -10388,7 +10388,7 @@
     </row>
     <row r="19" spans="1:81">
       <c r="A19" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B19">
         <v>2027</v>
@@ -10396,326 +10396,326 @@
     </row>
     <row r="20" spans="1:81">
       <c r="A20" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B20">
-        <f>IF(B$13&gt;=$B$19,0,B15)</f>
+        <f t="shared" ref="B20:AG20" si="3">IF(B$13&gt;=$B$19,0,B15)</f>
         <v>5.3308997197454321E-2</v>
       </c>
       <c r="C20">
-        <f>IF(C$13&gt;=$B$19,0,C15)</f>
+        <f t="shared" si="3"/>
         <v>7.4040273885353225E-2</v>
       </c>
       <c r="D20">
-        <f>IF(D$13&gt;=$B$19,0,D15)</f>
+        <f t="shared" si="3"/>
         <v>7.7001884840767351E-2</v>
       </c>
       <c r="E20">
-        <f>IF(E$13&gt;=$B$19,0,E15)</f>
+        <f t="shared" si="3"/>
         <v>7.9963495796181491E-2</v>
       </c>
       <c r="F20">
-        <f>IF(F$13&gt;=$B$19,0,F15)</f>
+        <f t="shared" si="3"/>
         <v>8.2925106751595618E-2</v>
       </c>
       <c r="G20">
-        <f>IF(G$13&gt;=$B$19,0,G15)</f>
+        <f t="shared" si="3"/>
         <v>8.884832866242387E-2</v>
       </c>
       <c r="H20">
-        <f>IF(H$13&gt;=$B$19,0,H15)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="I20">
-        <f>IF(I$13&gt;=$B$19,0,I15)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J20">
-        <f>IF(J$13&gt;=$B$19,0,J15)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="K20">
-        <f>IF(K$13&gt;=$B$19,0,K15)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L20">
-        <f>IF(L$13&gt;=$B$19,0,L15)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="M20">
-        <f>IF(M$13&gt;=$B$19,0,M15)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="N20">
-        <f>IF(N$13&gt;=$B$19,0,N15)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="O20">
-        <f>IF(O$13&gt;=$B$19,0,O15)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P20">
-        <f>IF(P$13&gt;=$B$19,0,P15)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="Q20">
-        <f>IF(Q$13&gt;=$B$19,0,Q15)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="R20">
-        <f>IF(R$13&gt;=$B$19,0,R15)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="S20">
-        <f>IF(S$13&gt;=$B$19,0,S15)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="T20">
-        <f>IF(T$13&gt;=$B$19,0,T15)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="U20">
-        <f>IF(U$13&gt;=$B$19,0,U15)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="V20">
-        <f>IF(V$13&gt;=$B$19,0,V15)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="W20">
-        <f>IF(W$13&gt;=$B$19,0,W15)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="X20">
-        <f>IF(X$13&gt;=$B$19,0,X15)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="Y20">
-        <f>IF(Y$13&gt;=$B$19,0,Y15)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="Z20">
-        <f>IF(Z$13&gt;=$B$19,0,Z15)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA20">
-        <f>IF(AA$13&gt;=$B$19,0,AA15)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AB20">
-        <f>IF(AB$13&gt;=$B$19,0,AB15)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AC20">
-        <f>IF(AC$13&gt;=$B$19,0,AC15)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AD20">
-        <f>IF(AD$13&gt;=$B$19,0,AD15)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AE20">
-        <f>IF(AE$13&gt;=$B$19,0,AE15)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AF20">
-        <f>IF(AF$13&gt;=$B$19,0,AF15)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AG20">
-        <f>IF(AG$13&gt;=$B$19,0,AG15)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AH20">
-        <f>IF(AH$13&gt;=$B$19,0,AH15)</f>
+        <f t="shared" ref="AH20:BM20" si="4">IF(AH$13&gt;=$B$19,0,AH15)</f>
         <v>0</v>
       </c>
       <c r="AI20">
-        <f>IF(AI$13&gt;=$B$19,0,AI15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AJ20">
-        <f>IF(AJ$13&gt;=$B$19,0,AJ15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AK20">
-        <f>IF(AK$13&gt;=$B$19,0,AK15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AL20">
-        <f>IF(AL$13&gt;=$B$19,0,AL15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AM20">
-        <f>IF(AM$13&gt;=$B$19,0,AM15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AN20">
-        <f>IF(AN$13&gt;=$B$19,0,AN15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AO20">
-        <f>IF(AO$13&gt;=$B$19,0,AO15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AP20">
-        <f>IF(AP$13&gt;=$B$19,0,AP15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AQ20">
-        <f>IF(AQ$13&gt;=$B$19,0,AQ15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AR20">
-        <f>IF(AR$13&gt;=$B$19,0,AR15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AS20">
-        <f>IF(AS$13&gt;=$B$19,0,AS15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AT20">
-        <f>IF(AT$13&gt;=$B$19,0,AT15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AU20">
-        <f>IF(AU$13&gt;=$B$19,0,AU15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AV20">
-        <f>IF(AV$13&gt;=$B$19,0,AV15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AW20">
-        <f>IF(AW$13&gt;=$B$19,0,AW15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AX20">
-        <f>IF(AX$13&gt;=$B$19,0,AX15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AY20">
-        <f>IF(AY$13&gt;=$B$19,0,AY15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AZ20">
-        <f>IF(AZ$13&gt;=$B$19,0,AZ15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="BA20">
-        <f>IF(BA$13&gt;=$B$19,0,BA15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="BB20">
-        <f>IF(BB$13&gt;=$B$19,0,BB15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="BC20">
-        <f>IF(BC$13&gt;=$B$19,0,BC15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="BD20">
-        <f>IF(BD$13&gt;=$B$19,0,BD15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="BE20">
-        <f>IF(BE$13&gt;=$B$19,0,BE15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="BF20">
-        <f>IF(BF$13&gt;=$B$19,0,BF15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="BG20">
-        <f>IF(BG$13&gt;=$B$19,0,BG15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="BH20">
-        <f>IF(BH$13&gt;=$B$19,0,BH15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="BI20">
-        <f>IF(BI$13&gt;=$B$19,0,BI15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="BJ20">
-        <f>IF(BJ$13&gt;=$B$19,0,BJ15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="BK20">
-        <f>IF(BK$13&gt;=$B$19,0,BK15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="BL20">
-        <f>IF(BL$13&gt;=$B$19,0,BL15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="BM20">
-        <f>IF(BM$13&gt;=$B$19,0,BM15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="BN20">
-        <f>IF(BN$13&gt;=$B$19,0,BN15)</f>
+        <f t="shared" ref="BN20:CC20" si="5">IF(BN$13&gt;=$B$19,0,BN15)</f>
         <v>0</v>
       </c>
       <c r="BO20">
-        <f>IF(BO$13&gt;=$B$19,0,BO15)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="BP20">
-        <f>IF(BP$13&gt;=$B$19,0,BP15)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="BQ20">
-        <f>IF(BQ$13&gt;=$B$19,0,BQ15)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="BR20">
-        <f>IF(BR$13&gt;=$B$19,0,BR15)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="BS20">
-        <f>IF(BS$13&gt;=$B$19,0,BS15)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="BT20">
-        <f>IF(BT$13&gt;=$B$19,0,BT15)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="BU20">
-        <f>IF(BU$13&gt;=$B$19,0,BU15)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="BV20">
-        <f>IF(BV$13&gt;=$B$19,0,BV15)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="BW20">
-        <f>IF(BW$13&gt;=$B$19,0,BW15)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="BX20">
-        <f>IF(BX$13&gt;=$B$19,0,BX15)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="BY20">
-        <f>IF(BY$13&gt;=$B$19,0,BY15)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="BZ20">
-        <f>IF(BZ$13&gt;=$B$19,0,BZ15)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="CA20">
-        <f>IF(CA$13&gt;=$B$19,0,CA15)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="CB20">
-        <f>IF(CB$13&gt;=$B$19,0,CB15)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="CC20">
-        <f>IF(CC$13&gt;=$B$19,0,CC15)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -10727,10 +10727,10 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{289D588D-DCC6-46C7-B1AC-54C9D46C0AE1}">
   <dimension ref="A1:CI26"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:87">
@@ -11923,17 +11923,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="A25:A26"/>
     <mergeCell ref="A15:A16"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A7:A8"/>
     <mergeCell ref="A9:A10"/>
     <mergeCell ref="A11:A12"/>
     <mergeCell ref="A13:A14"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A25:A26"/>
   </mergeCells>
   <phoneticPr fontId="26" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11947,10 +11947,10 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:CC61"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="19.7109375" customWidth="1"/>
-    <col min="2" max="2" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.7265625" customWidth="1"/>
+    <col min="2" max="2" width="20.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:81">
@@ -26990,10 +26990,10 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:CC61"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:81">
@@ -42033,10 +42033,10 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B61"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="14.28515625" style="11" customWidth="1"/>
+    <col min="2" max="2" width="14.26953125" style="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -42534,12 +42534,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E59C87379D9A4242BB3A95F198D6F941" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="07a235b40ffe2d9a960bde50f6511605">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="40f4d404-d193-41dc-bb72-733c1e774208" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="485fc8e6f691b86ce0aee9b7e82feca0" ns2:_="">
     <xsd:import namespace="40f4d404-d193-41dc-bb72-733c1e774208"/>
@@ -42683,6 +42677,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -42693,15 +42693,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD26A6D2-559B-4381-A873-3D2325889C28}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7715CECE-326A-4BF6-A74C-9A54CD69F51D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -42719,6 +42710,15 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD26A6D2-559B-4381-A873-3D2325889C28}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4E4DC507-1B00-4182-8466-350123371AC7}">
   <ds:schemaRefs>

</xml_diff>